<commit_message>
docs(sprint0): add backlog scoring, release plan, and burndown chart
Fill in the README backlog scoring table, capacity, 3-sprint release plan, and Scrum Master. Set up burndown.xlsx for 3 sprints with ideal, planned, and actual remaining lines.
</commit_message>
<xml_diff>
--- a/burndown.xlsx
+++ b/burndown.xlsx
@@ -1,37 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://msudenver-my.sharepoint.com/personal/tmota_msudenver_edu/Documents/Teaching/Courses/__24SCS3250_SE/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\CS3250\26FCS3250-002-prj-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7397B228-E7AA-634C-96A5-F3624B942EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF420D8-878A-4B72-89F1-21EAC2FE53E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1180" yWindow="1500" windowWidth="27240" windowHeight="15020" xr2:uid="{7A4C5A10-B1D5-9946-8D6C-7E3C0798020F}"/>
+    <workbookView xWindow="1410" yWindow="1450" windowWidth="28800" windowHeight="15370" xr2:uid="{7A4C5A10-B1D5-9946-8D6C-7E3C0798020F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Sheet1!$C$1:$G$1</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Sheet1!$C$2:$G$2</definedName>
-    <definedName name="_xlchart.v1.10" hidden="1">Sheet1!$C$3:$G$3</definedName>
-    <definedName name="_xlchart.v1.11" hidden="1">Sheet1!$C$1:$G$1</definedName>
-    <definedName name="_xlchart.v1.12" hidden="1">Sheet1!$C$2:$G$2</definedName>
-    <definedName name="_xlchart.v1.13" hidden="1">Sheet1!$C$3:$G$3</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Sheet1!$C$3:$G$3</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Sheet1!$C$4:$G$4</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$C$1:$G$1</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$C$2:$G$2</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$C$3:$G$3</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$C$4:$G$4</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">Sheet1!$C$1:$G$1</definedName>
-    <definedName name="_xlchart.v1.9" hidden="1">Sheet1!$C$2:$G$2</definedName>
-  </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -52,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Sprint 1</t>
   </si>
@@ -63,22 +47,19 @@
     <t>Sprint 3</t>
   </si>
   <si>
-    <t>Sprint 4</t>
-  </si>
-  <si>
-    <t>Sprint 5</t>
-  </si>
-  <si>
     <t>Planned</t>
   </si>
   <si>
     <t>Actual</t>
   </si>
   <si>
-    <t>Remaining</t>
+    <t>Actual remaining</t>
   </si>
   <si>
     <t>Start</t>
+  </si>
+  <si>
+    <t>Planned remaining</t>
   </si>
   <si>
     <t>Ideal</t>
@@ -160,7 +141,7 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -224,13 +205,8 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Project's</a:t>
+              <a:t>CampusEats Sprint Burndown</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Title</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -288,47 +264,38 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$1:$G$1</c:f>
+              <c:f>Sheet1!$B$1:$E$1</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Start</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Sprint 1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>Sprint 2</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>Sprint 3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Sprint 4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Sprint 5</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$2:$G$2</c:f>
+              <c:f>Sheet1!$B$2:$E$2</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>75</c:v>
-                </c:pt>
+                <c:ptCount val="4"/>
                 <c:pt idx="1">
-                  <c:v>60</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>80</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>40</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -357,48 +324,30 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet1!$C$1:$G$1</c:f>
+              <c:f>Sheet1!$B$1:$E$1</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
+                  <c:v>Start</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>Sprint 1</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>Sprint 2</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>Sprint 3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Sprint 4</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Sprint 5</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$3:$G$3</c:f>
+              <c:f>Sheet1!$B$3:$E$3</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
-                <c:pt idx="0">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>65</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>40</c:v>
-                </c:pt>
+                <c:ptCount val="4"/>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -427,39 +376,48 @@
           <c:idx val="2"/>
           <c:order val="2"/>
           <c:tx>
-            <c:v>Ideal Burndown</c:v>
+            <c:v>Planned remaining</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent3"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$4:$G$4</c:f>
+              <c:f>Sheet1!$B$4:$E$4</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>175</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>140</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="4">
                   <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
@@ -476,40 +434,49 @@
           <c:idx val="3"/>
           <c:order val="3"/>
           <c:tx>
-            <c:v>Remaining Effort</c:v>
+            <c:v>Actual remaining</c:v>
           </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent4"/>
+                <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$5:$G$5</c:f>
+              <c:f>Sheet1!$B$5:$E$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>200</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>155</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>90</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>#N/A</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -518,6 +485,65 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000007-3427-6247-871D-448016BD94EB}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>Ideal</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$6:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17.3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>8.6999999999999993</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-3427-6247-871D-448016BD94EB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -696,6 +722,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -703,7 +730,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1287,13 +1313,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>29936</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>178708</xdr:rowOff>
@@ -1325,9 +1351,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1365,7 +1391,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1471,7 +1497,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1613,7 +1639,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1621,16 +1647,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46ADD8F6-D520-684C-80D6-92D618A9A1CC}">
-  <dimension ref="A1:G5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="10.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="11.6640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="19" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B1" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>0</v>
@@ -1641,106 +1668,86 @@
       <c r="E1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>3</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3">
-        <v>75</v>
+        <v>10</v>
       </c>
       <c r="D2" s="3">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="E2" s="3">
-        <v>80</v>
-      </c>
-      <c r="F2" s="3">
-        <v>40</v>
-      </c>
-      <c r="G2" s="3">
-        <v>40</v>
+        <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="4">
-        <v>50</v>
-      </c>
-      <c r="D3" s="4">
-        <v>45</v>
-      </c>
-      <c r="E3" s="4">
-        <v>65</v>
-      </c>
-      <c r="F3" s="4">
-        <v>50</v>
-      </c>
-      <c r="G3" s="4">
-        <v>40</v>
-      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3"/>
+        <v>7</v>
+      </c>
+      <c r="B4" s="3">
+        <f>B5</f>
+        <v>26</v>
+      </c>
       <c r="C4" s="3">
-        <f>B5-C2</f>
-        <v>175</v>
+        <f>B4-C2</f>
+        <v>16</v>
       </c>
       <c r="D4" s="3">
-        <f t="shared" ref="D4:G4" si="0">C5-D2</f>
-        <v>140</v>
+        <f>C4-D2</f>
+        <v>8</v>
       </c>
       <c r="E4" s="3">
-        <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="F4" s="3">
-        <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="G4" s="3">
-        <f t="shared" si="0"/>
+        <f>D4-E2</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>250</v>
-      </c>
-      <c r="C5" s="4">
-        <f>B5-C3</f>
-        <v>200</v>
-      </c>
-      <c r="D5" s="4">
-        <f t="shared" ref="D5:G5" si="1">C5-D3</f>
-        <v>155</v>
-      </c>
-      <c r="E5" s="4">
-        <f t="shared" si="1"/>
-        <v>90</v>
-      </c>
-      <c r="F5" s="4">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="G5" s="4">
-        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="C5" s="4" t="e">
+        <f>IF(C3="",NA(),B5-C3)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D5" s="4" t="e">
+        <f>IF(D3="",NA(),C5-D3)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E5" s="4" t="e">
+        <f>IF(E3="",NA(),D5-E3)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3">
+        <v>17.3</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="E6" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>